<commit_message>
fix report, add dynamic update, add fields
</commit_message>
<xml_diff>
--- a/spring/ConstructorApp/src/main/resources/reportTemplate.xlsx
+++ b/spring/ConstructorApp/src/main/resources/reportTemplate.xlsx
@@ -8,16 +8,16 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\shats\IdeaProjects\constructor-reductor\spring\ConstructorApp\src\main\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6FCBB8DA-F456-4D30-B7CC-E4FF67F94C02}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BE34338C-A56E-4098-B6CD-F7482C23A9CF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="4995" yWindow="2895" windowWidth="21600" windowHeight="11295" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="КП" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="__xlnm_Print_Area" localSheetId="0">КП!$A$1:$K$85</definedName>
-    <definedName name="Excel_BuiltIn_Print_Area" localSheetId="0">КП!$A$1:$K$85</definedName>
+    <definedName name="__xlnm_Print_Area" localSheetId="0">КП!$A$1:$K$84</definedName>
+    <definedName name="Excel_BuiltIn_Print_Area" localSheetId="0">КП!$A$1:$K$84</definedName>
     <definedName name="FFF">NA()</definedName>
     <definedName name="GF">NA()</definedName>
     <definedName name="GFA">NA()</definedName>
@@ -57,7 +57,7 @@
     <definedName name="KKK">NA()</definedName>
     <definedName name="RRR">NA()</definedName>
     <definedName name="SSS">NA()</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">КП!$A$1:$K$88</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">КП!$A$1:$K$87</definedName>
     <definedName name="Типоразмеры">NA()</definedName>
   </definedNames>
   <calcPr calcId="191029" iterateDelta="1E-4"/>
@@ -76,7 +76,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="76" uniqueCount="55">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="75" uniqueCount="54">
   <si>
     <t xml:space="preserve"> </t>
   </si>
@@ -280,9 +280,6 @@
     <t>5. Гарантия 24 месяца.</t>
   </si>
   <si>
-    <t>Данное предложение действительно в течение 5 дней!!</t>
-  </si>
-  <si>
     <t xml:space="preserve">                               </t>
   </si>
   <si>
@@ -310,7 +307,7 @@
     <numFmt numFmtId="165" formatCode="#,##0\ _₽"/>
     <numFmt numFmtId="166" formatCode="#,##0.00\ _₽"/>
   </numFmts>
-  <fonts count="25" x14ac:knownFonts="1">
+  <fonts count="24" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color indexed="8"/>
@@ -461,15 +458,6 @@
       <color indexed="8"/>
       <name val="Calibri"/>
       <family val="2"/>
-    </font>
-    <font>
-      <b/>
-      <i/>
-      <u/>
-      <sz val="12"/>
-      <color indexed="16"/>
-      <name val="Times New Roman"/>
-      <family val="1"/>
     </font>
     <font>
       <sz val="12"/>
@@ -927,9 +915,9 @@
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="23" fillId="0" borderId="0" applyBorder="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="0" applyBorder="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="105">
+  <cellXfs count="104">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1" applyProtection="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1" applyProtection="1">
@@ -979,11 +967,11 @@
     <xf numFmtId="0" fontId="18" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="23" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1"/>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1"/>
     <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1" applyProtection="1"/>
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1" applyProtection="1"/>
     <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="15" fillId="3" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1"/>
@@ -1007,15 +995,12 @@
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="49" fontId="20" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="21" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1" applyProtection="1"/>
-    <xf numFmtId="49" fontId="22" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="49" fontId="20" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1" applyProtection="1"/>
+    <xf numFmtId="49" fontId="21" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="49" fontId="22" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1"/>
-    <xf numFmtId="49" fontId="22" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="49" fontId="21" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1"/>
+    <xf numFmtId="49" fontId="21" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="49" fontId="15" fillId="3" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
@@ -1024,12 +1009,138 @@
     <xf numFmtId="49" fontId="15" fillId="3" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="left"/>
     </xf>
+    <xf numFmtId="49" fontId="21" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="4" borderId="30" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="4" borderId="31" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="14" fillId="4" borderId="32" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="14" fillId="4" borderId="33" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="2" borderId="28" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="14" fillId="2" borderId="29" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="14" fillId="2" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="15" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="2" borderId="19" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="2" borderId="24" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="2" borderId="20" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="2" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="2" borderId="25" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="2" borderId="26" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="2" borderId="20" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="2" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="2" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="2" borderId="25" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="2" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="2" borderId="26" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="2" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="2" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="15" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="15" fillId="0" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="2" fontId="16" fillId="3" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="16" fillId="3" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="15" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="15" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="15" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="15" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="15" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="15" fillId="0" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="15" fillId="0" borderId="19" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1039,18 +1150,12 @@
     <xf numFmtId="0" fontId="15" fillId="0" borderId="20" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="15" fillId="0" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="15" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="15" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1063,18 +1168,9 @@
     <xf numFmtId="165" fontId="15" fillId="0" borderId="20" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="165" fontId="15" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="165" fontId="15" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="165" fontId="15" fillId="0" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="17" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center"/>
     </xf>
@@ -1089,117 +1185,6 @@
     </xf>
     <xf numFmtId="2" fontId="16" fillId="3" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="15" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="15" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="15" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="15" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="16" fillId="3" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="16" fillId="3" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="2" borderId="19" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="2" borderId="24" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="2" borderId="20" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="2" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="2" borderId="25" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="2" borderId="26" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="2" borderId="20" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="2" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="2" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="2" borderId="25" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="2" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="2" borderId="26" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="2" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="2" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="22" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="4" borderId="30" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="4" borderId="31" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="3" fontId="14" fillId="4" borderId="32" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="3" fontId="14" fillId="4" borderId="33" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="2" borderId="28" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="14" fillId="2" borderId="29" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="166" fontId="14" fillId="2" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="15" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -1445,13 +1430,13 @@
     <xdr:from>
       <xdr:col>10</xdr:col>
       <xdr:colOff>409575</xdr:colOff>
-      <xdr:row>43</xdr:row>
+      <xdr:row>42</xdr:row>
       <xdr:rowOff>47625</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>10</xdr:col>
       <xdr:colOff>619125</xdr:colOff>
-      <xdr:row>44</xdr:row>
+      <xdr:row>43</xdr:row>
       <xdr:rowOff>85725</xdr:rowOff>
     </xdr:to>
     <xdr:sp macro="" textlink="">
@@ -1516,13 +1501,13 @@
     <xdr:from>
       <xdr:col>10</xdr:col>
       <xdr:colOff>409575</xdr:colOff>
-      <xdr:row>84</xdr:row>
+      <xdr:row>83</xdr:row>
       <xdr:rowOff>95250</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>10</xdr:col>
       <xdr:colOff>619125</xdr:colOff>
-      <xdr:row>85</xdr:row>
+      <xdr:row>84</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:to>
     <xdr:sp macro="" textlink="">
@@ -1587,13 +1572,13 @@
     <xdr:from>
       <xdr:col>10</xdr:col>
       <xdr:colOff>409575</xdr:colOff>
-      <xdr:row>84</xdr:row>
+      <xdr:row>83</xdr:row>
       <xdr:rowOff>95250</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>10</xdr:col>
       <xdr:colOff>619125</xdr:colOff>
-      <xdr:row>85</xdr:row>
+      <xdr:row>84</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:to>
     <xdr:sp macro="" textlink="">
@@ -1658,13 +1643,13 @@
     <xdr:from>
       <xdr:col>10</xdr:col>
       <xdr:colOff>409575</xdr:colOff>
-      <xdr:row>84</xdr:row>
+      <xdr:row>83</xdr:row>
       <xdr:rowOff>95250</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>10</xdr:col>
       <xdr:colOff>619125</xdr:colOff>
-      <xdr:row>85</xdr:row>
+      <xdr:row>84</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:to>
     <xdr:sp macro="" textlink="">
@@ -1729,13 +1714,13 @@
     <xdr:from>
       <xdr:col>10</xdr:col>
       <xdr:colOff>409575</xdr:colOff>
-      <xdr:row>84</xdr:row>
+      <xdr:row>83</xdr:row>
       <xdr:rowOff>95250</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>10</xdr:col>
       <xdr:colOff>619125</xdr:colOff>
-      <xdr:row>85</xdr:row>
+      <xdr:row>84</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:to>
     <xdr:sp macro="" textlink="">
@@ -1800,13 +1785,13 @@
     <xdr:from>
       <xdr:col>10</xdr:col>
       <xdr:colOff>409575</xdr:colOff>
-      <xdr:row>84</xdr:row>
+      <xdr:row>83</xdr:row>
       <xdr:rowOff>95250</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>10</xdr:col>
       <xdr:colOff>619125</xdr:colOff>
-      <xdr:row>85</xdr:row>
+      <xdr:row>84</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:to>
     <xdr:sp macro="" textlink="">
@@ -1871,13 +1856,13 @@
     <xdr:from>
       <xdr:col>10</xdr:col>
       <xdr:colOff>409575</xdr:colOff>
-      <xdr:row>84</xdr:row>
+      <xdr:row>83</xdr:row>
       <xdr:rowOff>95250</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>10</xdr:col>
       <xdr:colOff>619125</xdr:colOff>
-      <xdr:row>85</xdr:row>
+      <xdr:row>84</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:to>
     <xdr:sp macro="" textlink="">
@@ -1942,13 +1927,13 @@
     <xdr:from>
       <xdr:col>10</xdr:col>
       <xdr:colOff>409575</xdr:colOff>
-      <xdr:row>84</xdr:row>
+      <xdr:row>83</xdr:row>
       <xdr:rowOff>95250</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>10</xdr:col>
       <xdr:colOff>619125</xdr:colOff>
-      <xdr:row>85</xdr:row>
+      <xdr:row>84</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:to>
     <xdr:sp macro="" textlink="">
@@ -2013,13 +1998,13 @@
     <xdr:from>
       <xdr:col>10</xdr:col>
       <xdr:colOff>409575</xdr:colOff>
-      <xdr:row>81</xdr:row>
+      <xdr:row>80</xdr:row>
       <xdr:rowOff>76200</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>10</xdr:col>
       <xdr:colOff>619125</xdr:colOff>
-      <xdr:row>84</xdr:row>
+      <xdr:row>83</xdr:row>
       <xdr:rowOff>114300</xdr:rowOff>
     </xdr:to>
     <xdr:sp macro="" textlink="">
@@ -2084,13 +2069,13 @@
     <xdr:from>
       <xdr:col>10</xdr:col>
       <xdr:colOff>409575</xdr:colOff>
-      <xdr:row>81</xdr:row>
+      <xdr:row>80</xdr:row>
       <xdr:rowOff>76200</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>10</xdr:col>
       <xdr:colOff>619125</xdr:colOff>
-      <xdr:row>84</xdr:row>
+      <xdr:row>83</xdr:row>
       <xdr:rowOff>114300</xdr:rowOff>
     </xdr:to>
     <xdr:sp macro="" textlink="">
@@ -2155,13 +2140,13 @@
     <xdr:from>
       <xdr:col>10</xdr:col>
       <xdr:colOff>409575</xdr:colOff>
-      <xdr:row>81</xdr:row>
+      <xdr:row>80</xdr:row>
       <xdr:rowOff>76200</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>10</xdr:col>
       <xdr:colOff>619125</xdr:colOff>
-      <xdr:row>84</xdr:row>
+      <xdr:row>83</xdr:row>
       <xdr:rowOff>114300</xdr:rowOff>
     </xdr:to>
     <xdr:sp macro="" textlink="">
@@ -2226,13 +2211,13 @@
     <xdr:from>
       <xdr:col>10</xdr:col>
       <xdr:colOff>409575</xdr:colOff>
-      <xdr:row>81</xdr:row>
+      <xdr:row>80</xdr:row>
       <xdr:rowOff>76200</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>10</xdr:col>
       <xdr:colOff>619125</xdr:colOff>
-      <xdr:row>84</xdr:row>
+      <xdr:row>83</xdr:row>
       <xdr:rowOff>114300</xdr:rowOff>
     </xdr:to>
     <xdr:sp macro="" textlink="">
@@ -2297,13 +2282,13 @@
     <xdr:from>
       <xdr:col>10</xdr:col>
       <xdr:colOff>409575</xdr:colOff>
-      <xdr:row>81</xdr:row>
+      <xdr:row>80</xdr:row>
       <xdr:rowOff>76200</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>10</xdr:col>
       <xdr:colOff>619125</xdr:colOff>
-      <xdr:row>84</xdr:row>
+      <xdr:row>83</xdr:row>
       <xdr:rowOff>114300</xdr:rowOff>
     </xdr:to>
     <xdr:sp macro="" textlink="">
@@ -2368,13 +2353,13 @@
     <xdr:from>
       <xdr:col>10</xdr:col>
       <xdr:colOff>409575</xdr:colOff>
-      <xdr:row>81</xdr:row>
+      <xdr:row>80</xdr:row>
       <xdr:rowOff>76200</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>10</xdr:col>
       <xdr:colOff>619125</xdr:colOff>
-      <xdr:row>84</xdr:row>
+      <xdr:row>83</xdr:row>
       <xdr:rowOff>114300</xdr:rowOff>
     </xdr:to>
     <xdr:sp macro="" textlink="">
@@ -2439,13 +2424,13 @@
     <xdr:from>
       <xdr:col>10</xdr:col>
       <xdr:colOff>409575</xdr:colOff>
-      <xdr:row>81</xdr:row>
+      <xdr:row>80</xdr:row>
       <xdr:rowOff>76200</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>10</xdr:col>
       <xdr:colOff>619125</xdr:colOff>
-      <xdr:row>84</xdr:row>
+      <xdr:row>83</xdr:row>
       <xdr:rowOff>114300</xdr:rowOff>
     </xdr:to>
     <xdr:sp macro="" textlink="">
@@ -2510,13 +2495,13 @@
     <xdr:from>
       <xdr:col>10</xdr:col>
       <xdr:colOff>409575</xdr:colOff>
-      <xdr:row>81</xdr:row>
+      <xdr:row>80</xdr:row>
       <xdr:rowOff>76200</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>10</xdr:col>
       <xdr:colOff>619125</xdr:colOff>
-      <xdr:row>84</xdr:row>
+      <xdr:row>83</xdr:row>
       <xdr:rowOff>114300</xdr:rowOff>
     </xdr:to>
     <xdr:sp macro="" textlink="">
@@ -2581,13 +2566,13 @@
     <xdr:from>
       <xdr:col>10</xdr:col>
       <xdr:colOff>409575</xdr:colOff>
-      <xdr:row>81</xdr:row>
+      <xdr:row>80</xdr:row>
       <xdr:rowOff>76200</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>10</xdr:col>
       <xdr:colOff>619125</xdr:colOff>
-      <xdr:row>84</xdr:row>
+      <xdr:row>83</xdr:row>
       <xdr:rowOff>114300</xdr:rowOff>
     </xdr:to>
     <xdr:sp macro="" textlink="">
@@ -2652,13 +2637,13 @@
     <xdr:from>
       <xdr:col>10</xdr:col>
       <xdr:colOff>409575</xdr:colOff>
-      <xdr:row>81</xdr:row>
+      <xdr:row>80</xdr:row>
       <xdr:rowOff>76200</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>10</xdr:col>
       <xdr:colOff>619125</xdr:colOff>
-      <xdr:row>84</xdr:row>
+      <xdr:row>83</xdr:row>
       <xdr:rowOff>114300</xdr:rowOff>
     </xdr:to>
     <xdr:sp macro="" textlink="">
@@ -2723,13 +2708,13 @@
     <xdr:from>
       <xdr:col>10</xdr:col>
       <xdr:colOff>409575</xdr:colOff>
-      <xdr:row>81</xdr:row>
+      <xdr:row>80</xdr:row>
       <xdr:rowOff>76200</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>10</xdr:col>
       <xdr:colOff>619125</xdr:colOff>
-      <xdr:row>84</xdr:row>
+      <xdr:row>83</xdr:row>
       <xdr:rowOff>114300</xdr:rowOff>
     </xdr:to>
     <xdr:sp macro="" textlink="">
@@ -2794,13 +2779,13 @@
     <xdr:from>
       <xdr:col>10</xdr:col>
       <xdr:colOff>409575</xdr:colOff>
-      <xdr:row>81</xdr:row>
+      <xdr:row>80</xdr:row>
       <xdr:rowOff>76200</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>10</xdr:col>
       <xdr:colOff>619125</xdr:colOff>
-      <xdr:row>84</xdr:row>
+      <xdr:row>83</xdr:row>
       <xdr:rowOff>114300</xdr:rowOff>
     </xdr:to>
     <xdr:sp macro="" textlink="">
@@ -2865,13 +2850,13 @@
     <xdr:from>
       <xdr:col>10</xdr:col>
       <xdr:colOff>409575</xdr:colOff>
-      <xdr:row>81</xdr:row>
+      <xdr:row>80</xdr:row>
       <xdr:rowOff>76200</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>10</xdr:col>
       <xdr:colOff>619125</xdr:colOff>
-      <xdr:row>84</xdr:row>
+      <xdr:row>83</xdr:row>
       <xdr:rowOff>114300</xdr:rowOff>
     </xdr:to>
     <xdr:sp macro="" textlink="">
@@ -2936,13 +2921,13 @@
     <xdr:from>
       <xdr:col>10</xdr:col>
       <xdr:colOff>409575</xdr:colOff>
-      <xdr:row>81</xdr:row>
+      <xdr:row>80</xdr:row>
       <xdr:rowOff>76200</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>10</xdr:col>
       <xdr:colOff>619125</xdr:colOff>
-      <xdr:row>84</xdr:row>
+      <xdr:row>83</xdr:row>
       <xdr:rowOff>114300</xdr:rowOff>
     </xdr:to>
     <xdr:sp macro="" textlink="">
@@ -3007,13 +2992,13 @@
     <xdr:from>
       <xdr:col>10</xdr:col>
       <xdr:colOff>409575</xdr:colOff>
-      <xdr:row>81</xdr:row>
+      <xdr:row>80</xdr:row>
       <xdr:rowOff>76200</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>10</xdr:col>
       <xdr:colOff>619125</xdr:colOff>
-      <xdr:row>84</xdr:row>
+      <xdr:row>83</xdr:row>
       <xdr:rowOff>114300</xdr:rowOff>
     </xdr:to>
     <xdr:sp macro="" textlink="">
@@ -3078,13 +3063,13 @@
     <xdr:from>
       <xdr:col>10</xdr:col>
       <xdr:colOff>409575</xdr:colOff>
-      <xdr:row>81</xdr:row>
+      <xdr:row>80</xdr:row>
       <xdr:rowOff>76200</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>10</xdr:col>
       <xdr:colOff>619125</xdr:colOff>
-      <xdr:row>84</xdr:row>
+      <xdr:row>83</xdr:row>
       <xdr:rowOff>114300</xdr:rowOff>
     </xdr:to>
     <xdr:sp macro="" textlink="">
@@ -3149,13 +3134,13 @@
     <xdr:from>
       <xdr:col>10</xdr:col>
       <xdr:colOff>409575</xdr:colOff>
-      <xdr:row>81</xdr:row>
+      <xdr:row>80</xdr:row>
       <xdr:rowOff>76200</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>10</xdr:col>
       <xdr:colOff>619125</xdr:colOff>
-      <xdr:row>84</xdr:row>
+      <xdr:row>83</xdr:row>
       <xdr:rowOff>114300</xdr:rowOff>
     </xdr:to>
     <xdr:sp macro="" textlink="">
@@ -3220,13 +3205,13 @@
     <xdr:from>
       <xdr:col>10</xdr:col>
       <xdr:colOff>409575</xdr:colOff>
-      <xdr:row>81</xdr:row>
+      <xdr:row>80</xdr:row>
       <xdr:rowOff>76200</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>10</xdr:col>
       <xdr:colOff>619125</xdr:colOff>
-      <xdr:row>84</xdr:row>
+      <xdr:row>83</xdr:row>
       <xdr:rowOff>114300</xdr:rowOff>
     </xdr:to>
     <xdr:sp macro="" textlink="">
@@ -3291,13 +3276,13 @@
     <xdr:from>
       <xdr:col>10</xdr:col>
       <xdr:colOff>409575</xdr:colOff>
-      <xdr:row>81</xdr:row>
+      <xdr:row>80</xdr:row>
       <xdr:rowOff>76200</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>10</xdr:col>
       <xdr:colOff>619125</xdr:colOff>
-      <xdr:row>84</xdr:row>
+      <xdr:row>83</xdr:row>
       <xdr:rowOff>114300</xdr:rowOff>
     </xdr:to>
     <xdr:sp macro="" textlink="">
@@ -3362,13 +3347,13 @@
     <xdr:from>
       <xdr:col>10</xdr:col>
       <xdr:colOff>409575</xdr:colOff>
-      <xdr:row>81</xdr:row>
+      <xdr:row>80</xdr:row>
       <xdr:rowOff>76200</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>10</xdr:col>
       <xdr:colOff>619125</xdr:colOff>
-      <xdr:row>84</xdr:row>
+      <xdr:row>83</xdr:row>
       <xdr:rowOff>114300</xdr:rowOff>
     </xdr:to>
     <xdr:sp macro="" textlink="">
@@ -3433,13 +3418,13 @@
     <xdr:from>
       <xdr:col>10</xdr:col>
       <xdr:colOff>409575</xdr:colOff>
-      <xdr:row>81</xdr:row>
+      <xdr:row>80</xdr:row>
       <xdr:rowOff>76200</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>10</xdr:col>
       <xdr:colOff>619125</xdr:colOff>
-      <xdr:row>84</xdr:row>
+      <xdr:row>83</xdr:row>
       <xdr:rowOff>114300</xdr:rowOff>
     </xdr:to>
     <xdr:sp macro="" textlink="">
@@ -3504,13 +3489,13 @@
     <xdr:from>
       <xdr:col>10</xdr:col>
       <xdr:colOff>409575</xdr:colOff>
-      <xdr:row>81</xdr:row>
+      <xdr:row>80</xdr:row>
       <xdr:rowOff>76200</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>10</xdr:col>
       <xdr:colOff>619125</xdr:colOff>
-      <xdr:row>84</xdr:row>
+      <xdr:row>83</xdr:row>
       <xdr:rowOff>114300</xdr:rowOff>
     </xdr:to>
     <xdr:sp macro="" textlink="">
@@ -3575,13 +3560,13 @@
     <xdr:from>
       <xdr:col>10</xdr:col>
       <xdr:colOff>409575</xdr:colOff>
-      <xdr:row>81</xdr:row>
+      <xdr:row>80</xdr:row>
       <xdr:rowOff>76200</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>10</xdr:col>
       <xdr:colOff>619125</xdr:colOff>
-      <xdr:row>84</xdr:row>
+      <xdr:row>83</xdr:row>
       <xdr:rowOff>114300</xdr:rowOff>
     </xdr:to>
     <xdr:sp macro="" textlink="">
@@ -3646,13 +3631,13 @@
     <xdr:from>
       <xdr:col>10</xdr:col>
       <xdr:colOff>409575</xdr:colOff>
-      <xdr:row>81</xdr:row>
+      <xdr:row>80</xdr:row>
       <xdr:rowOff>76200</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>10</xdr:col>
       <xdr:colOff>619125</xdr:colOff>
-      <xdr:row>84</xdr:row>
+      <xdr:row>83</xdr:row>
       <xdr:rowOff>114300</xdr:rowOff>
     </xdr:to>
     <xdr:sp macro="" textlink="">
@@ -3717,13 +3702,13 @@
     <xdr:from>
       <xdr:col>10</xdr:col>
       <xdr:colOff>409575</xdr:colOff>
-      <xdr:row>81</xdr:row>
+      <xdr:row>80</xdr:row>
       <xdr:rowOff>76200</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>10</xdr:col>
       <xdr:colOff>619125</xdr:colOff>
-      <xdr:row>84</xdr:row>
+      <xdr:row>83</xdr:row>
       <xdr:rowOff>114300</xdr:rowOff>
     </xdr:to>
     <xdr:sp macro="" textlink="">
@@ -3788,13 +3773,13 @@
     <xdr:from>
       <xdr:col>10</xdr:col>
       <xdr:colOff>409575</xdr:colOff>
-      <xdr:row>81</xdr:row>
+      <xdr:row>80</xdr:row>
       <xdr:rowOff>76200</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>10</xdr:col>
       <xdr:colOff>619125</xdr:colOff>
-      <xdr:row>84</xdr:row>
+      <xdr:row>83</xdr:row>
       <xdr:rowOff>114300</xdr:rowOff>
     </xdr:to>
     <xdr:sp macro="" textlink="">
@@ -3859,13 +3844,13 @@
     <xdr:from>
       <xdr:col>10</xdr:col>
       <xdr:colOff>409575</xdr:colOff>
-      <xdr:row>81</xdr:row>
+      <xdr:row>80</xdr:row>
       <xdr:rowOff>76200</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>10</xdr:col>
       <xdr:colOff>619125</xdr:colOff>
-      <xdr:row>84</xdr:row>
+      <xdr:row>83</xdr:row>
       <xdr:rowOff>114300</xdr:rowOff>
     </xdr:to>
     <xdr:sp macro="" textlink="">
@@ -3930,13 +3915,13 @@
     <xdr:from>
       <xdr:col>10</xdr:col>
       <xdr:colOff>409575</xdr:colOff>
-      <xdr:row>81</xdr:row>
+      <xdr:row>80</xdr:row>
       <xdr:rowOff>76200</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>10</xdr:col>
       <xdr:colOff>619125</xdr:colOff>
-      <xdr:row>84</xdr:row>
+      <xdr:row>83</xdr:row>
       <xdr:rowOff>114300</xdr:rowOff>
     </xdr:to>
     <xdr:sp macro="" textlink="">
@@ -4001,13 +3986,13 @@
     <xdr:from>
       <xdr:col>10</xdr:col>
       <xdr:colOff>409575</xdr:colOff>
-      <xdr:row>81</xdr:row>
+      <xdr:row>80</xdr:row>
       <xdr:rowOff>76200</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>10</xdr:col>
       <xdr:colOff>619125</xdr:colOff>
-      <xdr:row>84</xdr:row>
+      <xdr:row>83</xdr:row>
       <xdr:rowOff>114300</xdr:rowOff>
     </xdr:to>
     <xdr:sp macro="" textlink="">
@@ -4072,13 +4057,13 @@
     <xdr:from>
       <xdr:col>10</xdr:col>
       <xdr:colOff>409575</xdr:colOff>
-      <xdr:row>81</xdr:row>
+      <xdr:row>80</xdr:row>
       <xdr:rowOff>76200</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>10</xdr:col>
       <xdr:colOff>619125</xdr:colOff>
-      <xdr:row>84</xdr:row>
+      <xdr:row>83</xdr:row>
       <xdr:rowOff>114300</xdr:rowOff>
     </xdr:to>
     <xdr:sp macro="" textlink="">
@@ -4143,13 +4128,13 @@
     <xdr:from>
       <xdr:col>10</xdr:col>
       <xdr:colOff>409575</xdr:colOff>
-      <xdr:row>81</xdr:row>
+      <xdr:row>80</xdr:row>
       <xdr:rowOff>76200</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>10</xdr:col>
       <xdr:colOff>619125</xdr:colOff>
-      <xdr:row>84</xdr:row>
+      <xdr:row>83</xdr:row>
       <xdr:rowOff>114300</xdr:rowOff>
     </xdr:to>
     <xdr:sp macro="" textlink="">
@@ -4214,13 +4199,13 @@
     <xdr:from>
       <xdr:col>10</xdr:col>
       <xdr:colOff>752475</xdr:colOff>
-      <xdr:row>62</xdr:row>
+      <xdr:row>61</xdr:row>
       <xdr:rowOff>47625</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>10</xdr:col>
       <xdr:colOff>962025</xdr:colOff>
-      <xdr:row>63</xdr:row>
+      <xdr:row>62</xdr:row>
       <xdr:rowOff>85725</xdr:rowOff>
     </xdr:to>
     <xdr:sp macro="" textlink="">
@@ -4285,13 +4270,13 @@
     <xdr:from>
       <xdr:col>10</xdr:col>
       <xdr:colOff>409575</xdr:colOff>
-      <xdr:row>75</xdr:row>
+      <xdr:row>74</xdr:row>
       <xdr:rowOff>47625</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>10</xdr:col>
       <xdr:colOff>619125</xdr:colOff>
-      <xdr:row>76</xdr:row>
+      <xdr:row>75</xdr:row>
       <xdr:rowOff>85725</xdr:rowOff>
     </xdr:to>
     <xdr:sp macro="" textlink="">
@@ -4740,7 +4725,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:K107"/>
+  <dimension ref="A1:K106"/>
   <sheetFormatPr defaultColWidth="8.5703125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="9" style="1" customWidth="1"/>
@@ -4777,7 +4762,7 @@
     </row>
     <row r="6" spans="1:11" x14ac:dyDescent="0.25">
       <c r="D6" s="1" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
     </row>
     <row r="7" spans="1:11" ht="17.25" customHeight="1" x14ac:dyDescent="0.25"/>
@@ -4791,8 +4776,8 @@
       <c r="I8" s="8" t="s">
         <v>4</v>
       </c>
-      <c r="J8" s="78"/>
-      <c r="K8" s="78"/>
+      <c r="J8" s="56"/>
+      <c r="K8" s="56"/>
     </row>
     <row r="9" spans="1:11" ht="19.5" x14ac:dyDescent="0.25">
       <c r="C9" s="6"/>
@@ -4804,15 +4789,15 @@
       <c r="I9" s="8" t="s">
         <v>5</v>
       </c>
-      <c r="J9" s="78"/>
-      <c r="K9" s="78"/>
+      <c r="J9" s="56"/>
+      <c r="K9" s="56"/>
     </row>
     <row r="10" spans="1:11" ht="21" x14ac:dyDescent="0.35">
-      <c r="C10" s="79" t="s">
+      <c r="C10" s="57" t="s">
         <v>6</v>
       </c>
-      <c r="D10" s="79"/>
-      <c r="E10" s="79"/>
+      <c r="D10" s="57"/>
+      <c r="E10" s="57"/>
       <c r="F10" s="9"/>
       <c r="G10" s="10" t="s">
         <v>7</v>
@@ -4834,80 +4819,80 @@
       <c r="K11" s="6"/>
     </row>
     <row r="12" spans="1:11" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B12" s="80" t="s">
+      <c r="B12" s="58" t="s">
         <v>8</v>
       </c>
-      <c r="C12" s="82" t="s">
+      <c r="C12" s="60" t="s">
         <v>9</v>
       </c>
-      <c r="D12" s="83"/>
-      <c r="E12" s="86" t="s">
+      <c r="D12" s="61"/>
+      <c r="E12" s="64" t="s">
         <v>10</v>
       </c>
-      <c r="F12" s="87"/>
-      <c r="G12" s="88"/>
+      <c r="F12" s="65"/>
+      <c r="G12" s="66"/>
       <c r="H12" s="29" t="s">
         <v>11</v>
       </c>
-      <c r="I12" s="82" t="s">
+      <c r="I12" s="60" t="s">
         <v>12</v>
       </c>
-      <c r="J12" s="92"/>
+      <c r="J12" s="70"/>
     </row>
     <row r="13" spans="1:11" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B13" s="81"/>
-      <c r="C13" s="84"/>
-      <c r="D13" s="85"/>
-      <c r="E13" s="89"/>
-      <c r="F13" s="90"/>
-      <c r="G13" s="91"/>
+      <c r="B13" s="59"/>
+      <c r="C13" s="62"/>
+      <c r="D13" s="63"/>
+      <c r="E13" s="67"/>
+      <c r="F13" s="68"/>
+      <c r="G13" s="69"/>
       <c r="H13" s="30" t="s">
         <v>13</v>
       </c>
-      <c r="I13" s="84" t="str">
+      <c r="I13" s="62" t="str">
         <f>H13</f>
         <v>Юань ¥</v>
       </c>
-      <c r="J13" s="93"/>
+      <c r="J13" s="71"/>
     </row>
     <row r="14" spans="1:11" ht="16.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B14" s="95" t="s">
+      <c r="B14" s="46" t="s">
         <v>38</v>
       </c>
-      <c r="C14" s="96"/>
-      <c r="D14" s="96"/>
-      <c r="E14" s="96"/>
-      <c r="F14" s="96"/>
-      <c r="G14" s="96"/>
-      <c r="H14" s="96"/>
-      <c r="I14" s="97"/>
-      <c r="J14" s="98"/>
+      <c r="C14" s="47"/>
+      <c r="D14" s="47"/>
+      <c r="E14" s="47"/>
+      <c r="F14" s="47"/>
+      <c r="G14" s="47"/>
+      <c r="H14" s="47"/>
+      <c r="I14" s="48"/>
+      <c r="J14" s="49"/>
     </row>
     <row r="15" spans="1:11" ht="17.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B15" s="99" t="s">
+      <c r="B15" s="50" t="s">
         <v>39</v>
       </c>
-      <c r="C15" s="99"/>
-      <c r="D15" s="99"/>
-      <c r="E15" s="99"/>
-      <c r="F15" s="99"/>
-      <c r="G15" s="99"/>
-      <c r="H15" s="99"/>
-      <c r="I15" s="101"/>
-      <c r="J15" s="101"/>
+      <c r="C15" s="50"/>
+      <c r="D15" s="50"/>
+      <c r="E15" s="50"/>
+      <c r="F15" s="50"/>
+      <c r="G15" s="50"/>
+      <c r="H15" s="50"/>
+      <c r="I15" s="52"/>
+      <c r="J15" s="52"/>
     </row>
     <row r="16" spans="1:11" ht="17.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B16" s="100" t="s">
+      <c r="B16" s="51" t="s">
         <v>40</v>
       </c>
-      <c r="C16" s="100"/>
-      <c r="D16" s="100"/>
-      <c r="E16" s="100"/>
-      <c r="F16" s="100"/>
-      <c r="G16" s="100"/>
-      <c r="H16" s="100"/>
-      <c r="I16" s="102"/>
-      <c r="J16" s="102"/>
+      <c r="C16" s="51"/>
+      <c r="D16" s="51"/>
+      <c r="E16" s="51"/>
+      <c r="F16" s="51"/>
+      <c r="G16" s="51"/>
+      <c r="H16" s="51"/>
+      <c r="I16" s="53"/>
+      <c r="J16" s="53"/>
     </row>
     <row r="17" spans="2:11" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B17" s="15"/>
@@ -4921,17 +4906,17 @@
       <c r="J17" s="15"/>
     </row>
     <row r="18" spans="2:11" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B18" s="103" t="s">
+      <c r="B18" s="54" t="s">
         <v>41</v>
       </c>
-      <c r="C18" s="103"/>
-      <c r="D18" s="103"/>
-      <c r="E18" s="103"/>
-      <c r="F18" s="103"/>
-      <c r="G18" s="103"/>
-      <c r="H18" s="103"/>
-      <c r="I18" s="103"/>
-      <c r="J18" s="103"/>
+      <c r="C18" s="54"/>
+      <c r="D18" s="54"/>
+      <c r="E18" s="54"/>
+      <c r="F18" s="54"/>
+      <c r="G18" s="54"/>
+      <c r="H18" s="54"/>
+      <c r="I18" s="54"/>
+      <c r="J18" s="54"/>
     </row>
     <row r="19" spans="2:11" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B19" s="35"/>
@@ -4946,30 +4931,30 @@
       <c r="K19" s="36"/>
     </row>
     <row r="20" spans="2:11" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B20" s="104" t="s">
+      <c r="B20" s="55" t="s">
         <v>42</v>
       </c>
-      <c r="C20" s="104"/>
-      <c r="D20" s="104"/>
-      <c r="E20" s="104"/>
-      <c r="F20" s="104"/>
-      <c r="G20" s="104"/>
-      <c r="H20" s="104"/>
-      <c r="I20" s="104"/>
-      <c r="J20" s="104"/>
-      <c r="K20" s="104"/>
+      <c r="C20" s="55"/>
+      <c r="D20" s="55"/>
+      <c r="E20" s="55"/>
+      <c r="F20" s="55"/>
+      <c r="G20" s="55"/>
+      <c r="H20" s="55"/>
+      <c r="I20" s="55"/>
+      <c r="J20" s="55"/>
+      <c r="K20" s="55"/>
     </row>
     <row r="21" spans="2:11" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B21" s="104"/>
-      <c r="C21" s="104"/>
-      <c r="D21" s="104"/>
-      <c r="E21" s="104"/>
-      <c r="F21" s="104"/>
-      <c r="G21" s="104"/>
-      <c r="H21" s="104"/>
-      <c r="I21" s="104"/>
-      <c r="J21" s="104"/>
-      <c r="K21" s="104"/>
+      <c r="B21" s="55"/>
+      <c r="C21" s="55"/>
+      <c r="D21" s="55"/>
+      <c r="E21" s="55"/>
+      <c r="F21" s="55"/>
+      <c r="G21" s="55"/>
+      <c r="H21" s="55"/>
+      <c r="I21" s="55"/>
+      <c r="J21" s="55"/>
+      <c r="K21" s="55"/>
     </row>
     <row r="22" spans="2:11" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B22" s="34" t="s">
@@ -5066,9 +5051,7 @@
       <c r="K28" s="36"/>
     </row>
     <row r="29" spans="2:11" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B29" s="39" t="s">
-        <v>48</v>
-      </c>
+      <c r="B29" s="38"/>
       <c r="C29" s="36"/>
       <c r="D29" s="36"/>
       <c r="E29" s="36"/>
@@ -5092,7 +5075,7 @@
       <c r="K30" s="36"/>
     </row>
     <row r="31" spans="2:11" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B31" s="38"/>
+      <c r="B31" s="39"/>
       <c r="C31" s="36"/>
       <c r="D31" s="36"/>
       <c r="E31" s="36"/>
@@ -5104,9 +5087,11 @@
       <c r="K31" s="36"/>
     </row>
     <row r="32" spans="2:11" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B32" s="40"/>
-      <c r="C32" s="36"/>
-      <c r="D32" s="36"/>
+      <c r="B32" s="45" t="s">
+        <v>49</v>
+      </c>
+      <c r="C32" s="45"/>
+      <c r="D32" s="45"/>
       <c r="E32" s="36"/>
       <c r="F32" s="36"/>
       <c r="G32" s="36"/>
@@ -5116,11 +5101,11 @@
       <c r="K32" s="36"/>
     </row>
     <row r="33" spans="2:11" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B33" s="94" t="s">
+      <c r="B33" s="40" t="s">
         <v>50</v>
       </c>
-      <c r="C33" s="94"/>
-      <c r="D33" s="94"/>
+      <c r="C33" s="40"/>
+      <c r="D33" s="36"/>
       <c r="E33" s="36"/>
       <c r="F33" s="36"/>
       <c r="G33" s="36"/>
@@ -5130,10 +5115,10 @@
       <c r="K33" s="36"/>
     </row>
     <row r="34" spans="2:11" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B34" s="41" t="s">
+      <c r="B34" s="45" t="s">
         <v>51</v>
       </c>
-      <c r="C34" s="41"/>
+      <c r="C34" s="45"/>
       <c r="D34" s="36"/>
       <c r="E34" s="36"/>
       <c r="F34" s="36"/>
@@ -5144,10 +5129,10 @@
       <c r="K34" s="36"/>
     </row>
     <row r="35" spans="2:11" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B35" s="94" t="s">
+      <c r="B35" s="41" t="s">
         <v>52</v>
       </c>
-      <c r="C35" s="94"/>
+      <c r="C35" s="42"/>
       <c r="D35" s="36"/>
       <c r="E35" s="36"/>
       <c r="F35" s="36"/>
@@ -5158,10 +5143,8 @@
       <c r="K35" s="36"/>
     </row>
     <row r="36" spans="2:11" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B36" s="42" t="s">
-        <v>53</v>
-      </c>
-      <c r="C36" s="43"/>
+      <c r="B36" s="38"/>
+      <c r="C36" s="36"/>
       <c r="D36" s="36"/>
       <c r="E36" s="36"/>
       <c r="F36" s="36"/>
@@ -5171,10 +5154,12 @@
       <c r="J36" s="36"/>
       <c r="K36" s="36"/>
     </row>
-    <row r="37" spans="2:11" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="37" spans="2:11" ht="29.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B37" s="38"/>
       <c r="C37" s="36"/>
-      <c r="D37" s="36"/>
+      <c r="D37" s="36" t="s">
+        <v>48</v>
+      </c>
       <c r="E37" s="36"/>
       <c r="F37" s="36"/>
       <c r="G37" s="36"/>
@@ -5183,614 +5168,601 @@
       <c r="J37" s="36"/>
       <c r="K37" s="36"/>
     </row>
-    <row r="38" spans="2:11" ht="29.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B38" s="38"/>
-      <c r="C38" s="36"/>
-      <c r="D38" s="36" t="s">
-        <v>49</v>
-      </c>
-      <c r="E38" s="36"/>
-      <c r="F38" s="36"/>
-      <c r="G38" s="36"/>
-      <c r="H38" s="36"/>
-      <c r="I38" s="36"/>
-      <c r="J38" s="36"/>
-      <c r="K38" s="36"/>
+    <row r="38" spans="2:11" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="D38"/>
     </row>
     <row r="39" spans="2:11" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="D39"/>
-    </row>
-    <row r="40" spans="2:11" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B40" s="21"/>
-      <c r="C40" s="21"/>
-      <c r="D40" s="22"/>
-      <c r="I40" s="23"/>
-    </row>
-    <row r="41" spans="2:11" ht="16.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3"/>
-    <row r="42" spans="2:11" ht="37.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B42" s="46"/>
-      <c r="C42" s="76"/>
-      <c r="D42" s="77"/>
-      <c r="E42" s="68"/>
-      <c r="F42" s="51"/>
-      <c r="G42" s="69"/>
-      <c r="H42" s="72"/>
-      <c r="I42" s="74"/>
-      <c r="J42" s="59"/>
+      <c r="B39" s="21"/>
+      <c r="C39" s="21"/>
+      <c r="D39" s="22"/>
+      <c r="I39" s="23"/>
+    </row>
+    <row r="40" spans="2:11" ht="16.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3"/>
+    <row r="41" spans="2:11" ht="37.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B41" s="72"/>
+      <c r="C41" s="74"/>
+      <c r="D41" s="75"/>
+      <c r="E41" s="76"/>
+      <c r="F41" s="77"/>
+      <c r="G41" s="78"/>
+      <c r="H41" s="82"/>
+      <c r="I41" s="84"/>
+      <c r="J41" s="85"/>
+    </row>
+    <row r="42" spans="2:11" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B42" s="73"/>
+      <c r="C42" s="13" t="s">
+        <v>14</v>
+      </c>
+      <c r="D42" s="13" t="s">
+        <v>15</v>
+      </c>
+      <c r="E42" s="79"/>
+      <c r="F42" s="80"/>
+      <c r="G42" s="81"/>
+      <c r="H42" s="83"/>
+      <c r="I42" s="86"/>
+      <c r="J42" s="87"/>
     </row>
     <row r="43" spans="2:11" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B43" s="47"/>
-      <c r="C43" s="13" t="s">
+      <c r="B43" s="73"/>
+      <c r="C43" s="14" t="s">
+        <v>16</v>
+      </c>
+      <c r="D43" s="24"/>
+      <c r="E43" s="79"/>
+      <c r="F43" s="80"/>
+      <c r="G43" s="81"/>
+      <c r="H43" s="83"/>
+      <c r="I43" s="86"/>
+      <c r="J43" s="87"/>
+    </row>
+    <row r="44" spans="2:11" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B44" s="73"/>
+      <c r="C44" s="14" t="s">
+        <v>17</v>
+      </c>
+      <c r="D44" s="16"/>
+      <c r="E44" s="79"/>
+      <c r="F44" s="80"/>
+      <c r="G44" s="81"/>
+      <c r="H44" s="83"/>
+      <c r="I44" s="86"/>
+      <c r="J44" s="87"/>
+    </row>
+    <row r="45" spans="2:11" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B45" s="73"/>
+      <c r="C45" s="14" t="s">
+        <v>18</v>
+      </c>
+      <c r="D45" s="17"/>
+      <c r="E45" s="79"/>
+      <c r="F45" s="80"/>
+      <c r="G45" s="81"/>
+      <c r="H45" s="83"/>
+      <c r="I45" s="86"/>
+      <c r="J45" s="87"/>
+    </row>
+    <row r="46" spans="2:11" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B46" s="73"/>
+      <c r="C46" s="14" t="s">
+        <v>19</v>
+      </c>
+      <c r="D46" s="17"/>
+      <c r="E46" s="79"/>
+      <c r="F46" s="80"/>
+      <c r="G46" s="81"/>
+      <c r="H46" s="83"/>
+      <c r="I46" s="86"/>
+      <c r="J46" s="87"/>
+    </row>
+    <row r="47" spans="2:11" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B47" s="73"/>
+      <c r="C47" s="14" t="s">
+        <v>20</v>
+      </c>
+      <c r="D47" s="18"/>
+      <c r="E47" s="79"/>
+      <c r="F47" s="80"/>
+      <c r="G47" s="81"/>
+      <c r="H47" s="83"/>
+      <c r="I47" s="86"/>
+      <c r="J47" s="87"/>
+    </row>
+    <row r="48" spans="2:11" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B48" s="73"/>
+      <c r="C48" s="14" t="s">
+        <v>21</v>
+      </c>
+      <c r="D48" s="19" t="s">
+        <v>22</v>
+      </c>
+      <c r="E48" s="79"/>
+      <c r="F48" s="80"/>
+      <c r="G48" s="81"/>
+      <c r="H48" s="83"/>
+      <c r="I48" s="86"/>
+      <c r="J48" s="87"/>
+    </row>
+    <row r="49" spans="2:10" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B49" s="73"/>
+      <c r="C49" s="14" t="s">
+        <v>23</v>
+      </c>
+      <c r="D49" s="16" t="s">
+        <v>24</v>
+      </c>
+      <c r="E49" s="79"/>
+      <c r="F49" s="80"/>
+      <c r="G49" s="81"/>
+      <c r="H49" s="83"/>
+      <c r="I49" s="86"/>
+      <c r="J49" s="87"/>
+    </row>
+    <row r="50" spans="2:10" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B50" s="73"/>
+      <c r="C50" s="14" t="s">
+        <v>25</v>
+      </c>
+      <c r="D50" s="16"/>
+      <c r="E50" s="79"/>
+      <c r="F50" s="80"/>
+      <c r="G50" s="81"/>
+      <c r="H50" s="83"/>
+      <c r="I50" s="86"/>
+      <c r="J50" s="87"/>
+    </row>
+    <row r="51" spans="2:10" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B51" s="73"/>
+      <c r="C51" s="14" t="s">
+        <v>26</v>
+      </c>
+      <c r="D51" s="16"/>
+      <c r="E51" s="79"/>
+      <c r="F51" s="80"/>
+      <c r="G51" s="81"/>
+      <c r="H51" s="83"/>
+      <c r="I51" s="86"/>
+      <c r="J51" s="87"/>
+    </row>
+    <row r="52" spans="2:10" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B52" s="73"/>
+      <c r="C52" s="14" t="s">
+        <v>27</v>
+      </c>
+      <c r="D52" s="16" t="s">
+        <v>28</v>
+      </c>
+      <c r="E52" s="79"/>
+      <c r="F52" s="80"/>
+      <c r="G52" s="81"/>
+      <c r="H52" s="83"/>
+      <c r="I52" s="86"/>
+      <c r="J52" s="87"/>
+    </row>
+    <row r="53" spans="2:10" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B53" s="73"/>
+      <c r="C53" s="14" t="s">
+        <v>29</v>
+      </c>
+      <c r="D53" s="16"/>
+      <c r="E53" s="79"/>
+      <c r="F53" s="80"/>
+      <c r="G53" s="81"/>
+      <c r="H53" s="83"/>
+      <c r="I53" s="86"/>
+      <c r="J53" s="87"/>
+    </row>
+    <row r="54" spans="2:10" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B54" s="73"/>
+      <c r="C54" s="14" t="s">
+        <v>30</v>
+      </c>
+      <c r="D54" s="16"/>
+      <c r="E54" s="79"/>
+      <c r="F54" s="80"/>
+      <c r="G54" s="81"/>
+      <c r="H54" s="83"/>
+      <c r="I54" s="86"/>
+      <c r="J54" s="87"/>
+    </row>
+    <row r="55" spans="2:10" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B55" s="73"/>
+      <c r="C55" s="14" t="s">
+        <v>31</v>
+      </c>
+      <c r="D55" s="16"/>
+      <c r="E55" s="79"/>
+      <c r="F55" s="80"/>
+      <c r="G55" s="81"/>
+      <c r="H55" s="83"/>
+      <c r="I55" s="86"/>
+      <c r="J55" s="87"/>
+    </row>
+    <row r="56" spans="2:10" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B56" s="73"/>
+      <c r="C56" s="14" t="s">
+        <v>32</v>
+      </c>
+      <c r="D56" s="16"/>
+      <c r="E56" s="79"/>
+      <c r="F56" s="80"/>
+      <c r="G56" s="81"/>
+      <c r="H56" s="83"/>
+      <c r="I56" s="86"/>
+      <c r="J56" s="87"/>
+    </row>
+    <row r="57" spans="2:10" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B57" s="73"/>
+      <c r="C57" s="14" t="s">
+        <v>33</v>
+      </c>
+      <c r="D57" s="17"/>
+      <c r="E57" s="79"/>
+      <c r="F57" s="80"/>
+      <c r="G57" s="81"/>
+      <c r="H57" s="83"/>
+      <c r="I57" s="86"/>
+      <c r="J57" s="87"/>
+    </row>
+    <row r="58" spans="2:10" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B58" s="73"/>
+      <c r="C58" s="27"/>
+      <c r="D58" s="43"/>
+      <c r="E58" s="79"/>
+      <c r="F58" s="80"/>
+      <c r="G58" s="81"/>
+      <c r="H58" s="83"/>
+      <c r="I58" s="86"/>
+      <c r="J58" s="87"/>
+    </row>
+    <row r="59" spans="2:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B59" s="31"/>
+      <c r="C59" s="32"/>
+      <c r="D59" s="28"/>
+      <c r="E59" s="88"/>
+      <c r="F59" s="88"/>
+      <c r="G59" s="88"/>
+      <c r="H59" s="28"/>
+      <c r="I59" s="88"/>
+      <c r="J59" s="88"/>
+    </row>
+    <row r="60" spans="2:10" ht="36.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B60" s="72"/>
+      <c r="C60" s="100"/>
+      <c r="D60" s="101"/>
+      <c r="E60" s="76"/>
+      <c r="F60" s="77"/>
+      <c r="G60" s="78"/>
+      <c r="H60" s="82"/>
+      <c r="I60" s="84"/>
+      <c r="J60" s="85"/>
+    </row>
+    <row r="61" spans="2:10" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="B61" s="73"/>
+      <c r="C61" s="20" t="s">
         <v>14</v>
       </c>
-      <c r="D43" s="13" t="s">
+      <c r="D61" s="20" t="s">
         <v>15</v>
       </c>
-      <c r="E43" s="70"/>
-      <c r="F43" s="54"/>
-      <c r="G43" s="71"/>
-      <c r="H43" s="73"/>
-      <c r="I43" s="75"/>
-      <c r="J43" s="61"/>
-    </row>
-    <row r="44" spans="2:11" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B44" s="47"/>
-      <c r="C44" s="14" t="s">
+      <c r="E61" s="79"/>
+      <c r="F61" s="80"/>
+      <c r="G61" s="81"/>
+      <c r="H61" s="83"/>
+      <c r="I61" s="86"/>
+      <c r="J61" s="87"/>
+    </row>
+    <row r="62" spans="2:10" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="B62" s="73"/>
+      <c r="C62" s="14" t="s">
+        <v>17</v>
+      </c>
+      <c r="D62" s="16"/>
+      <c r="E62" s="79"/>
+      <c r="F62" s="80"/>
+      <c r="G62" s="81"/>
+      <c r="H62" s="83"/>
+      <c r="I62" s="86"/>
+      <c r="J62" s="87"/>
+    </row>
+    <row r="63" spans="2:10" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="B63" s="73"/>
+      <c r="C63" s="14" t="s">
+        <v>18</v>
+      </c>
+      <c r="D63" s="17"/>
+      <c r="E63" s="79"/>
+      <c r="F63" s="80"/>
+      <c r="G63" s="81"/>
+      <c r="H63" s="83"/>
+      <c r="I63" s="86"/>
+      <c r="J63" s="87"/>
+    </row>
+    <row r="64" spans="2:10" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="B64" s="73"/>
+      <c r="C64" s="14" t="s">
+        <v>34</v>
+      </c>
+      <c r="D64" s="16"/>
+      <c r="E64" s="79"/>
+      <c r="F64" s="80"/>
+      <c r="G64" s="81"/>
+      <c r="H64" s="83"/>
+      <c r="I64" s="86"/>
+      <c r="J64" s="87"/>
+    </row>
+    <row r="65" spans="2:10" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="B65" s="73"/>
+      <c r="C65" s="14" t="s">
+        <v>35</v>
+      </c>
+      <c r="D65" s="16"/>
+      <c r="E65" s="79"/>
+      <c r="F65" s="80"/>
+      <c r="G65" s="81"/>
+      <c r="H65" s="83"/>
+      <c r="I65" s="86"/>
+      <c r="J65" s="87"/>
+    </row>
+    <row r="66" spans="2:10" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="B66" s="73"/>
+      <c r="C66" s="14" t="s">
+        <v>21</v>
+      </c>
+      <c r="D66" s="19" t="s">
+        <v>22</v>
+      </c>
+      <c r="E66" s="79"/>
+      <c r="F66" s="80"/>
+      <c r="G66" s="81"/>
+      <c r="H66" s="83"/>
+      <c r="I66" s="86"/>
+      <c r="J66" s="87"/>
+    </row>
+    <row r="67" spans="2:10" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="B67" s="73"/>
+      <c r="C67" s="14" t="s">
+        <v>23</v>
+      </c>
+      <c r="D67" s="16" t="s">
+        <v>24</v>
+      </c>
+      <c r="E67" s="79"/>
+      <c r="F67" s="80"/>
+      <c r="G67" s="81"/>
+      <c r="H67" s="83"/>
+      <c r="I67" s="86"/>
+      <c r="J67" s="87"/>
+    </row>
+    <row r="68" spans="2:10" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="B68" s="73"/>
+      <c r="C68" s="14" t="s">
+        <v>36</v>
+      </c>
+      <c r="D68" s="16"/>
+      <c r="E68" s="79"/>
+      <c r="F68" s="80"/>
+      <c r="G68" s="81"/>
+      <c r="H68" s="83"/>
+      <c r="I68" s="86"/>
+      <c r="J68" s="87"/>
+    </row>
+    <row r="69" spans="2:10" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="B69" s="73"/>
+      <c r="C69" s="14" t="s">
+        <v>32</v>
+      </c>
+      <c r="D69" s="16"/>
+      <c r="E69" s="79"/>
+      <c r="F69" s="80"/>
+      <c r="G69" s="81"/>
+      <c r="H69" s="83"/>
+      <c r="I69" s="86"/>
+      <c r="J69" s="87"/>
+    </row>
+    <row r="70" spans="2:10" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="B70" s="73"/>
+      <c r="C70" s="14" t="s">
+        <v>37</v>
+      </c>
+      <c r="D70" s="17"/>
+      <c r="E70" s="79"/>
+      <c r="F70" s="80"/>
+      <c r="G70" s="81"/>
+      <c r="H70" s="83"/>
+      <c r="I70" s="86"/>
+      <c r="J70" s="87"/>
+    </row>
+    <row r="71" spans="2:10" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="B71" s="73"/>
+      <c r="C71" s="14"/>
+      <c r="D71" s="43"/>
+      <c r="E71" s="79"/>
+      <c r="F71" s="80"/>
+      <c r="G71" s="81"/>
+      <c r="H71" s="83"/>
+      <c r="I71" s="86"/>
+      <c r="J71" s="87"/>
+    </row>
+    <row r="72" spans="2:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B72" s="31"/>
+      <c r="C72" s="32"/>
+      <c r="D72" s="28"/>
+      <c r="E72" s="99"/>
+      <c r="F72" s="99"/>
+      <c r="G72" s="99"/>
+      <c r="H72" s="32"/>
+      <c r="I72" s="88"/>
+      <c r="J72" s="88"/>
+    </row>
+    <row r="73" spans="2:10" ht="36.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B73" s="89"/>
+      <c r="C73" s="102"/>
+      <c r="D73" s="103"/>
+      <c r="E73" s="91"/>
+      <c r="F73" s="77"/>
+      <c r="G73" s="92"/>
+      <c r="H73" s="95"/>
+      <c r="I73" s="97"/>
+      <c r="J73" s="85"/>
+    </row>
+    <row r="74" spans="2:10" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="B74" s="90"/>
+      <c r="C74" s="13" t="s">
+        <v>14</v>
+      </c>
+      <c r="D74" s="13" t="s">
+        <v>15</v>
+      </c>
+      <c r="E74" s="93"/>
+      <c r="F74" s="80"/>
+      <c r="G74" s="94"/>
+      <c r="H74" s="96"/>
+      <c r="I74" s="98"/>
+      <c r="J74" s="87"/>
+    </row>
+    <row r="75" spans="2:10" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="B75" s="90"/>
+      <c r="C75" s="14" t="s">
         <v>16</v>
       </c>
-      <c r="D44" s="24"/>
-      <c r="E44" s="70"/>
-      <c r="F44" s="54"/>
-      <c r="G44" s="71"/>
-      <c r="H44" s="73"/>
-      <c r="I44" s="75"/>
-      <c r="J44" s="61"/>
-    </row>
-    <row r="45" spans="2:11" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B45" s="47"/>
-      <c r="C45" s="14" t="s">
-        <v>17</v>
-      </c>
-      <c r="D45" s="16"/>
-      <c r="E45" s="70"/>
-      <c r="F45" s="54"/>
-      <c r="G45" s="71"/>
-      <c r="H45" s="73"/>
-      <c r="I45" s="75"/>
-      <c r="J45" s="61"/>
-    </row>
-    <row r="46" spans="2:11" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B46" s="47"/>
-      <c r="C46" s="14" t="s">
-        <v>18</v>
-      </c>
-      <c r="D46" s="17"/>
-      <c r="E46" s="70"/>
-      <c r="F46" s="54"/>
-      <c r="G46" s="71"/>
-      <c r="H46" s="73"/>
-      <c r="I46" s="75"/>
-      <c r="J46" s="61"/>
-    </row>
-    <row r="47" spans="2:11" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B47" s="47"/>
-      <c r="C47" s="14" t="s">
+      <c r="D75" s="24"/>
+      <c r="E75" s="93"/>
+      <c r="F75" s="80"/>
+      <c r="G75" s="94"/>
+      <c r="H75" s="96"/>
+      <c r="I75" s="98"/>
+      <c r="J75" s="87"/>
+    </row>
+    <row r="76" spans="2:10" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="B76" s="90"/>
+      <c r="C76" s="14" t="s">
         <v>19</v>
       </c>
-      <c r="D47" s="17"/>
-      <c r="E47" s="70"/>
-      <c r="F47" s="54"/>
-      <c r="G47" s="71"/>
-      <c r="H47" s="73"/>
-      <c r="I47" s="75"/>
-      <c r="J47" s="61"/>
-    </row>
-    <row r="48" spans="2:11" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B48" s="47"/>
-      <c r="C48" s="14" t="s">
-        <v>20</v>
-      </c>
-      <c r="D48" s="18"/>
-      <c r="E48" s="70"/>
-      <c r="F48" s="54"/>
-      <c r="G48" s="71"/>
-      <c r="H48" s="73"/>
-      <c r="I48" s="75"/>
-      <c r="J48" s="61"/>
-    </row>
-    <row r="49" spans="2:10" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B49" s="47"/>
-      <c r="C49" s="14" t="s">
-        <v>21</v>
-      </c>
-      <c r="D49" s="19" t="s">
-        <v>22</v>
-      </c>
-      <c r="E49" s="70"/>
-      <c r="F49" s="54"/>
-      <c r="G49" s="71"/>
-      <c r="H49" s="73"/>
-      <c r="I49" s="75"/>
-      <c r="J49" s="61"/>
-    </row>
-    <row r="50" spans="2:10" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B50" s="47"/>
-      <c r="C50" s="14" t="s">
-        <v>23</v>
-      </c>
-      <c r="D50" s="16" t="s">
-        <v>24</v>
-      </c>
-      <c r="E50" s="70"/>
-      <c r="F50" s="54"/>
-      <c r="G50" s="71"/>
-      <c r="H50" s="73"/>
-      <c r="I50" s="75"/>
-      <c r="J50" s="61"/>
-    </row>
-    <row r="51" spans="2:10" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B51" s="47"/>
-      <c r="C51" s="14" t="s">
+      <c r="D76" s="17"/>
+      <c r="E76" s="93"/>
+      <c r="F76" s="80"/>
+      <c r="G76" s="94"/>
+      <c r="H76" s="96"/>
+      <c r="I76" s="98"/>
+      <c r="J76" s="87"/>
+    </row>
+    <row r="77" spans="2:10" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="B77" s="90"/>
+      <c r="C77" s="14" t="s">
         <v>25</v>
       </c>
-      <c r="D51" s="16"/>
-      <c r="E51" s="70"/>
-      <c r="F51" s="54"/>
-      <c r="G51" s="71"/>
-      <c r="H51" s="73"/>
-      <c r="I51" s="75"/>
-      <c r="J51" s="61"/>
-    </row>
-    <row r="52" spans="2:10" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B52" s="47"/>
-      <c r="C52" s="14" t="s">
+      <c r="D77" s="16"/>
+      <c r="E77" s="93"/>
+      <c r="F77" s="80"/>
+      <c r="G77" s="94"/>
+      <c r="H77" s="96"/>
+      <c r="I77" s="98"/>
+      <c r="J77" s="87"/>
+    </row>
+    <row r="78" spans="2:10" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="B78" s="90"/>
+      <c r="C78" s="14" t="s">
         <v>26</v>
       </c>
-      <c r="D52" s="16"/>
-      <c r="E52" s="70"/>
-      <c r="F52" s="54"/>
-      <c r="G52" s="71"/>
-      <c r="H52" s="73"/>
-      <c r="I52" s="75"/>
-      <c r="J52" s="61"/>
-    </row>
-    <row r="53" spans="2:10" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B53" s="47"/>
-      <c r="C53" s="14" t="s">
+      <c r="D78" s="16"/>
+      <c r="E78" s="93"/>
+      <c r="F78" s="80"/>
+      <c r="G78" s="94"/>
+      <c r="H78" s="96"/>
+      <c r="I78" s="98"/>
+      <c r="J78" s="87"/>
+    </row>
+    <row r="79" spans="2:10" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="B79" s="90"/>
+      <c r="C79" s="14" t="s">
         <v>27</v>
       </c>
-      <c r="D53" s="16" t="s">
+      <c r="D79" s="16" t="s">
         <v>28</v>
       </c>
-      <c r="E53" s="70"/>
-      <c r="F53" s="54"/>
-      <c r="G53" s="71"/>
-      <c r="H53" s="73"/>
-      <c r="I53" s="75"/>
-      <c r="J53" s="61"/>
-    </row>
-    <row r="54" spans="2:10" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B54" s="47"/>
-      <c r="C54" s="14" t="s">
+      <c r="E79" s="93"/>
+      <c r="F79" s="80"/>
+      <c r="G79" s="94"/>
+      <c r="H79" s="96"/>
+      <c r="I79" s="98"/>
+      <c r="J79" s="87"/>
+    </row>
+    <row r="80" spans="2:10" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="B80" s="90"/>
+      <c r="C80" s="14" t="s">
         <v>29</v>
       </c>
-      <c r="D54" s="16"/>
-      <c r="E54" s="70"/>
-      <c r="F54" s="54"/>
-      <c r="G54" s="71"/>
-      <c r="H54" s="73"/>
-      <c r="I54" s="75"/>
-      <c r="J54" s="61"/>
-    </row>
-    <row r="55" spans="2:10" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B55" s="47"/>
-      <c r="C55" s="14" t="s">
+      <c r="D80" s="16"/>
+      <c r="E80" s="93"/>
+      <c r="F80" s="80"/>
+      <c r="G80" s="94"/>
+      <c r="H80" s="96"/>
+      <c r="I80" s="98"/>
+      <c r="J80" s="87"/>
+    </row>
+    <row r="81" spans="2:10" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="B81" s="90"/>
+      <c r="C81" s="14" t="s">
         <v>30</v>
       </c>
-      <c r="D55" s="16"/>
-      <c r="E55" s="70"/>
-      <c r="F55" s="54"/>
-      <c r="G55" s="71"/>
-      <c r="H55" s="73"/>
-      <c r="I55" s="75"/>
-      <c r="J55" s="61"/>
-    </row>
-    <row r="56" spans="2:10" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B56" s="47"/>
-      <c r="C56" s="14" t="s">
-        <v>31</v>
-      </c>
-      <c r="D56" s="16"/>
-      <c r="E56" s="70"/>
-      <c r="F56" s="54"/>
-      <c r="G56" s="71"/>
-      <c r="H56" s="73"/>
-      <c r="I56" s="75"/>
-      <c r="J56" s="61"/>
-    </row>
-    <row r="57" spans="2:10" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B57" s="47"/>
-      <c r="C57" s="14" t="s">
+      <c r="D81" s="16"/>
+      <c r="E81" s="93"/>
+      <c r="F81" s="80"/>
+      <c r="G81" s="94"/>
+      <c r="H81" s="96"/>
+      <c r="I81" s="98"/>
+      <c r="J81" s="87"/>
+    </row>
+    <row r="82" spans="2:10" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="B82" s="90"/>
+      <c r="C82" s="14" t="s">
         <v>32</v>
       </c>
-      <c r="D57" s="16"/>
-      <c r="E57" s="70"/>
-      <c r="F57" s="54"/>
-      <c r="G57" s="71"/>
-      <c r="H57" s="73"/>
-      <c r="I57" s="75"/>
-      <c r="J57" s="61"/>
-    </row>
-    <row r="58" spans="2:10" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B58" s="47"/>
-      <c r="C58" s="14" t="s">
+      <c r="D82" s="16"/>
+      <c r="E82" s="93"/>
+      <c r="F82" s="80"/>
+      <c r="G82" s="94"/>
+      <c r="H82" s="96"/>
+      <c r="I82" s="98"/>
+      <c r="J82" s="87"/>
+    </row>
+    <row r="83" spans="2:10" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="B83" s="90"/>
+      <c r="C83" s="14" t="s">
         <v>33</v>
       </c>
-      <c r="D58" s="17"/>
-      <c r="E58" s="70"/>
-      <c r="F58" s="54"/>
-      <c r="G58" s="71"/>
-      <c r="H58" s="73"/>
-      <c r="I58" s="75"/>
-      <c r="J58" s="61"/>
-    </row>
-    <row r="59" spans="2:10" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B59" s="47"/>
-      <c r="C59" s="27"/>
-      <c r="D59" s="44"/>
-      <c r="E59" s="70"/>
-      <c r="F59" s="54"/>
-      <c r="G59" s="71"/>
-      <c r="H59" s="73"/>
-      <c r="I59" s="75"/>
-      <c r="J59" s="61"/>
-    </row>
-    <row r="60" spans="2:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B60" s="31"/>
-      <c r="C60" s="32"/>
-      <c r="D60" s="28"/>
-      <c r="E60" s="62"/>
-      <c r="F60" s="62"/>
-      <c r="G60" s="62"/>
-      <c r="H60" s="28"/>
-      <c r="I60" s="62"/>
-      <c r="J60" s="62"/>
-    </row>
-    <row r="61" spans="2:10" ht="36.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B61" s="46"/>
-      <c r="C61" s="64"/>
-      <c r="D61" s="65"/>
-      <c r="E61" s="68"/>
-      <c r="F61" s="51"/>
-      <c r="G61" s="69"/>
-      <c r="H61" s="72"/>
-      <c r="I61" s="74"/>
-      <c r="J61" s="59"/>
-    </row>
-    <row r="62" spans="2:10" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="B62" s="47"/>
-      <c r="C62" s="20" t="s">
-        <v>14</v>
-      </c>
-      <c r="D62" s="20" t="s">
-        <v>15</v>
-      </c>
-      <c r="E62" s="70"/>
-      <c r="F62" s="54"/>
-      <c r="G62" s="71"/>
-      <c r="H62" s="73"/>
-      <c r="I62" s="75"/>
-      <c r="J62" s="61"/>
-    </row>
-    <row r="63" spans="2:10" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="B63" s="47"/>
-      <c r="C63" s="14" t="s">
-        <v>17</v>
-      </c>
-      <c r="D63" s="16"/>
-      <c r="E63" s="70"/>
-      <c r="F63" s="54"/>
-      <c r="G63" s="71"/>
-      <c r="H63" s="73"/>
-      <c r="I63" s="75"/>
-      <c r="J63" s="61"/>
-    </row>
-    <row r="64" spans="2:10" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="B64" s="47"/>
-      <c r="C64" s="14" t="s">
-        <v>18</v>
-      </c>
-      <c r="D64" s="17"/>
-      <c r="E64" s="70"/>
-      <c r="F64" s="54"/>
-      <c r="G64" s="71"/>
-      <c r="H64" s="73"/>
-      <c r="I64" s="75"/>
-      <c r="J64" s="61"/>
-    </row>
-    <row r="65" spans="2:10" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="B65" s="47"/>
-      <c r="C65" s="14" t="s">
-        <v>34</v>
-      </c>
-      <c r="D65" s="16"/>
-      <c r="E65" s="70"/>
-      <c r="F65" s="54"/>
-      <c r="G65" s="71"/>
-      <c r="H65" s="73"/>
-      <c r="I65" s="75"/>
-      <c r="J65" s="61"/>
-    </row>
-    <row r="66" spans="2:10" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="B66" s="47"/>
-      <c r="C66" s="14" t="s">
-        <v>35</v>
-      </c>
-      <c r="D66" s="16"/>
-      <c r="E66" s="70"/>
-      <c r="F66" s="54"/>
-      <c r="G66" s="71"/>
-      <c r="H66" s="73"/>
-      <c r="I66" s="75"/>
-      <c r="J66" s="61"/>
-    </row>
-    <row r="67" spans="2:10" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="B67" s="47"/>
-      <c r="C67" s="14" t="s">
-        <v>21</v>
-      </c>
-      <c r="D67" s="19" t="s">
-        <v>22</v>
-      </c>
-      <c r="E67" s="70"/>
-      <c r="F67" s="54"/>
-      <c r="G67" s="71"/>
-      <c r="H67" s="73"/>
-      <c r="I67" s="75"/>
-      <c r="J67" s="61"/>
-    </row>
-    <row r="68" spans="2:10" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="B68" s="47"/>
-      <c r="C68" s="14" t="s">
-        <v>23</v>
-      </c>
-      <c r="D68" s="16" t="s">
-        <v>24</v>
-      </c>
-      <c r="E68" s="70"/>
-      <c r="F68" s="54"/>
-      <c r="G68" s="71"/>
-      <c r="H68" s="73"/>
-      <c r="I68" s="75"/>
-      <c r="J68" s="61"/>
-    </row>
-    <row r="69" spans="2:10" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="B69" s="47"/>
-      <c r="C69" s="14" t="s">
-        <v>36</v>
-      </c>
-      <c r="D69" s="16"/>
-      <c r="E69" s="70"/>
-      <c r="F69" s="54"/>
-      <c r="G69" s="71"/>
-      <c r="H69" s="73"/>
-      <c r="I69" s="75"/>
-      <c r="J69" s="61"/>
-    </row>
-    <row r="70" spans="2:10" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="B70" s="47"/>
-      <c r="C70" s="14" t="s">
-        <v>32</v>
-      </c>
-      <c r="D70" s="16"/>
-      <c r="E70" s="70"/>
-      <c r="F70" s="54"/>
-      <c r="G70" s="71"/>
-      <c r="H70" s="73"/>
-      <c r="I70" s="75"/>
-      <c r="J70" s="61"/>
-    </row>
-    <row r="71" spans="2:10" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="B71" s="47"/>
-      <c r="C71" s="14" t="s">
-        <v>37</v>
-      </c>
-      <c r="D71" s="17"/>
-      <c r="E71" s="70"/>
-      <c r="F71" s="54"/>
-      <c r="G71" s="71"/>
-      <c r="H71" s="73"/>
-      <c r="I71" s="75"/>
-      <c r="J71" s="61"/>
-    </row>
-    <row r="72" spans="2:10" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="B72" s="47"/>
-      <c r="C72" s="14"/>
-      <c r="D72" s="44"/>
-      <c r="E72" s="70"/>
-      <c r="F72" s="54"/>
-      <c r="G72" s="71"/>
-      <c r="H72" s="73"/>
-      <c r="I72" s="75"/>
-      <c r="J72" s="61"/>
-    </row>
-    <row r="73" spans="2:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B73" s="31"/>
-      <c r="C73" s="32"/>
-      <c r="D73" s="28"/>
-      <c r="E73" s="63"/>
-      <c r="F73" s="63"/>
-      <c r="G73" s="63"/>
-      <c r="H73" s="32"/>
-      <c r="I73" s="62"/>
-      <c r="J73" s="62"/>
-    </row>
-    <row r="74" spans="2:10" ht="36.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B74" s="48"/>
-      <c r="C74" s="66"/>
-      <c r="D74" s="67"/>
-      <c r="E74" s="50"/>
-      <c r="F74" s="51"/>
-      <c r="G74" s="52"/>
-      <c r="H74" s="56"/>
-      <c r="I74" s="58"/>
-      <c r="J74" s="59"/>
-    </row>
-    <row r="75" spans="2:10" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="B75" s="49"/>
-      <c r="C75" s="13" t="s">
-        <v>14</v>
-      </c>
-      <c r="D75" s="13" t="s">
-        <v>15</v>
-      </c>
-      <c r="E75" s="53"/>
-      <c r="F75" s="54"/>
-      <c r="G75" s="55"/>
-      <c r="H75" s="57"/>
-      <c r="I75" s="60"/>
-      <c r="J75" s="61"/>
-    </row>
-    <row r="76" spans="2:10" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="B76" s="49"/>
-      <c r="C76" s="14" t="s">
-        <v>16</v>
-      </c>
-      <c r="D76" s="24"/>
-      <c r="E76" s="53"/>
-      <c r="F76" s="54"/>
-      <c r="G76" s="55"/>
-      <c r="H76" s="57"/>
-      <c r="I76" s="60"/>
-      <c r="J76" s="61"/>
-    </row>
-    <row r="77" spans="2:10" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="B77" s="49"/>
-      <c r="C77" s="14" t="s">
-        <v>19</v>
-      </c>
-      <c r="D77" s="17"/>
-      <c r="E77" s="53"/>
-      <c r="F77" s="54"/>
-      <c r="G77" s="55"/>
-      <c r="H77" s="57"/>
-      <c r="I77" s="60"/>
-      <c r="J77" s="61"/>
-    </row>
-    <row r="78" spans="2:10" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="B78" s="49"/>
-      <c r="C78" s="14" t="s">
-        <v>25</v>
-      </c>
-      <c r="D78" s="16"/>
-      <c r="E78" s="53"/>
-      <c r="F78" s="54"/>
-      <c r="G78" s="55"/>
-      <c r="H78" s="57"/>
-      <c r="I78" s="60"/>
-      <c r="J78" s="61"/>
-    </row>
-    <row r="79" spans="2:10" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="B79" s="49"/>
-      <c r="C79" s="14" t="s">
-        <v>26</v>
-      </c>
-      <c r="D79" s="16"/>
-      <c r="E79" s="53"/>
-      <c r="F79" s="54"/>
-      <c r="G79" s="55"/>
-      <c r="H79" s="57"/>
-      <c r="I79" s="60"/>
-      <c r="J79" s="61"/>
-    </row>
-    <row r="80" spans="2:10" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="B80" s="49"/>
-      <c r="C80" s="14" t="s">
-        <v>27</v>
-      </c>
-      <c r="D80" s="16" t="s">
-        <v>28</v>
-      </c>
-      <c r="E80" s="53"/>
-      <c r="F80" s="54"/>
-      <c r="G80" s="55"/>
-      <c r="H80" s="57"/>
-      <c r="I80" s="60"/>
-      <c r="J80" s="61"/>
-    </row>
-    <row r="81" spans="2:10" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="B81" s="49"/>
-      <c r="C81" s="14" t="s">
-        <v>29</v>
-      </c>
-      <c r="D81" s="16"/>
-      <c r="E81" s="53"/>
-      <c r="F81" s="54"/>
-      <c r="G81" s="55"/>
-      <c r="H81" s="57"/>
-      <c r="I81" s="60"/>
-      <c r="J81" s="61"/>
-    </row>
-    <row r="82" spans="2:10" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="B82" s="49"/>
-      <c r="C82" s="14" t="s">
-        <v>30</v>
-      </c>
-      <c r="D82" s="16"/>
-      <c r="E82" s="53"/>
-      <c r="F82" s="54"/>
-      <c r="G82" s="55"/>
-      <c r="H82" s="57"/>
-      <c r="I82" s="60"/>
-      <c r="J82" s="61"/>
-    </row>
-    <row r="83" spans="2:10" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="B83" s="49"/>
-      <c r="C83" s="14" t="s">
-        <v>32</v>
-      </c>
-      <c r="D83" s="16"/>
-      <c r="E83" s="53"/>
-      <c r="F83" s="54"/>
-      <c r="G83" s="55"/>
-      <c r="H83" s="57"/>
-      <c r="I83" s="60"/>
-      <c r="J83" s="61"/>
-    </row>
-    <row r="84" spans="2:10" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="B84" s="49"/>
-      <c r="C84" s="14" t="s">
-        <v>33</v>
-      </c>
-      <c r="D84" s="17"/>
-      <c r="E84" s="53"/>
-      <c r="F84" s="54"/>
-      <c r="G84" s="55"/>
-      <c r="H84" s="57"/>
-      <c r="I84" s="60"/>
-      <c r="J84" s="61"/>
-    </row>
-    <row r="85" spans="2:10" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B85" s="49"/>
-      <c r="C85" s="26"/>
-      <c r="D85" s="45"/>
-      <c r="E85" s="53"/>
-      <c r="F85" s="54"/>
-      <c r="G85" s="55"/>
-      <c r="H85" s="57"/>
-      <c r="I85" s="60"/>
-      <c r="J85" s="61"/>
-    </row>
-    <row r="86" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B86" s="25"/>
-      <c r="C86" s="28"/>
-      <c r="E86" s="28"/>
-      <c r="F86" s="28"/>
-      <c r="G86" s="28"/>
-      <c r="H86" s="28"/>
-      <c r="I86" s="28"/>
-      <c r="J86" s="28"/>
-    </row>
+      <c r="D83" s="17"/>
+      <c r="E83" s="93"/>
+      <c r="F83" s="80"/>
+      <c r="G83" s="94"/>
+      <c r="H83" s="96"/>
+      <c r="I83" s="98"/>
+      <c r="J83" s="87"/>
+    </row>
+    <row r="84" spans="2:10" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B84" s="90"/>
+      <c r="C84" s="26"/>
+      <c r="D84" s="44"/>
+      <c r="E84" s="93"/>
+      <c r="F84" s="80"/>
+      <c r="G84" s="94"/>
+      <c r="H84" s="96"/>
+      <c r="I84" s="98"/>
+      <c r="J84" s="87"/>
+    </row>
+    <row r="85" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B85" s="25"/>
+      <c r="C85" s="28"/>
+      <c r="E85" s="28"/>
+      <c r="F85" s="28"/>
+      <c r="G85" s="28"/>
+      <c r="H85" s="28"/>
+      <c r="I85" s="28"/>
+      <c r="J85" s="28"/>
+    </row>
+    <row r="96" spans="2:10" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="97" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="98" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="99" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25"/>
@@ -5801,12 +5773,38 @@
     <row r="104" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="105" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="106" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="107" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25"/>
   </sheetData>
   <sheetProtection selectLockedCells="1" selectUnlockedCells="1"/>
   <mergeCells count="38">
-    <mergeCell ref="B33:D33"/>
-    <mergeCell ref="B35:C35"/>
+    <mergeCell ref="B60:B71"/>
+    <mergeCell ref="B73:B84"/>
+    <mergeCell ref="E73:G84"/>
+    <mergeCell ref="H73:H84"/>
+    <mergeCell ref="I73:J84"/>
+    <mergeCell ref="I72:J72"/>
+    <mergeCell ref="E72:G72"/>
+    <mergeCell ref="C60:D60"/>
+    <mergeCell ref="C73:D73"/>
+    <mergeCell ref="E59:G59"/>
+    <mergeCell ref="I59:J59"/>
+    <mergeCell ref="E60:G71"/>
+    <mergeCell ref="H60:H71"/>
+    <mergeCell ref="I60:J71"/>
+    <mergeCell ref="B41:B58"/>
+    <mergeCell ref="C41:D41"/>
+    <mergeCell ref="E41:G58"/>
+    <mergeCell ref="H41:H58"/>
+    <mergeCell ref="I41:J58"/>
+    <mergeCell ref="J8:K8"/>
+    <mergeCell ref="J9:K9"/>
+    <mergeCell ref="C10:E10"/>
+    <mergeCell ref="B12:B13"/>
+    <mergeCell ref="C12:D13"/>
+    <mergeCell ref="E12:G13"/>
+    <mergeCell ref="I12:J12"/>
+    <mergeCell ref="I13:J13"/>
+    <mergeCell ref="B32:D32"/>
+    <mergeCell ref="B34:C34"/>
     <mergeCell ref="B14:H14"/>
     <mergeCell ref="I14:J14"/>
     <mergeCell ref="B15:H15"/>
@@ -5816,49 +5814,22 @@
     <mergeCell ref="B18:J18"/>
     <mergeCell ref="B20:K20"/>
     <mergeCell ref="B21:K21"/>
-    <mergeCell ref="J8:K8"/>
-    <mergeCell ref="J9:K9"/>
-    <mergeCell ref="C10:E10"/>
-    <mergeCell ref="B12:B13"/>
-    <mergeCell ref="C12:D13"/>
-    <mergeCell ref="E12:G13"/>
-    <mergeCell ref="I12:J12"/>
-    <mergeCell ref="I13:J13"/>
-    <mergeCell ref="B42:B59"/>
-    <mergeCell ref="C42:D42"/>
-    <mergeCell ref="E42:G59"/>
-    <mergeCell ref="H42:H59"/>
-    <mergeCell ref="I42:J59"/>
-    <mergeCell ref="E60:G60"/>
-    <mergeCell ref="I60:J60"/>
-    <mergeCell ref="E61:G72"/>
-    <mergeCell ref="H61:H72"/>
-    <mergeCell ref="I61:J72"/>
-    <mergeCell ref="B61:B72"/>
-    <mergeCell ref="B74:B85"/>
-    <mergeCell ref="E74:G85"/>
-    <mergeCell ref="H74:H85"/>
-    <mergeCell ref="I74:J85"/>
-    <mergeCell ref="I73:J73"/>
-    <mergeCell ref="E73:G73"/>
-    <mergeCell ref="C61:D61"/>
-    <mergeCell ref="C74:D74"/>
   </mergeCells>
   <dataValidations count="5">
     <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="H13" xr:uid="{00000000-0002-0000-0000-000000000000}">
       <formula1>"Руб.₽,Доллар $,Евро €,Юань ¥,"</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation allowBlank="1" showErrorMessage="1" sqref="D54 D52 D69:D72 B34" xr:uid="{00000000-0002-0000-0000-000001000000}"/>
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="D80 D53" xr:uid="{00000000-0002-0000-0000-000002000000}">
+    <dataValidation allowBlank="1" showErrorMessage="1" sqref="D53 D51 D68:D71 B33" xr:uid="{00000000-0002-0000-0000-000001000000}"/>
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="D79 D52" xr:uid="{00000000-0002-0000-0000-000002000000}">
       <formula1>"Да,Нет"</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation allowBlank="1" showErrorMessage="1" sqref="D46 D50:D51 D64 D68 D77:D79 D81" xr:uid="{00000000-0002-0000-0000-000005000000}">
+    <dataValidation allowBlank="1" showErrorMessage="1" sqref="D45 D49:D50 D63 D67 D76:D78 D80" xr:uid="{00000000-0002-0000-0000-000005000000}">
       <formula1>0</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="D49 D67" xr:uid="{00000000-0002-0000-0000-000006000000}">
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="D48 D66" xr:uid="{00000000-0002-0000-0000-000006000000}">
       <formula1>#REF!</formula1>
       <formula2>0</formula2>
     </dataValidation>

</xml_diff>